<commit_message>
fix: 回补 Dashboard 饿了么店铺数 2026-10-16
</commit_message>
<xml_diff>
--- a/data-dashboard/public/data/饿了么数据.xlsx
+++ b/data-dashboard/public/data/饿了么数据.xlsx
@@ -6140,7 +6140,7 @@
         <v>1766.09</v>
       </c>
       <c r="C357" t="n">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="D357" t="n">
         <v>8</v>
@@ -6156,7 +6156,7 @@
         <v>1769.04</v>
       </c>
       <c r="C358" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D358" t="n">
         <v>4</v>
@@ -6172,7 +6172,7 @@
         <v>1906</v>
       </c>
       <c r="C359" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D359" t="n">
         <v>7</v>
@@ -6204,7 +6204,7 @@
         <v>2242.11</v>
       </c>
       <c r="C361" t="n">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D361" t="n">
         <v>8</v>
@@ -6220,7 +6220,7 @@
         <v>1923.93</v>
       </c>
       <c r="C362" t="n">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D362" t="n">
         <v>6</v>
@@ -6236,7 +6236,7 @@
         <v>1895.55</v>
       </c>
       <c r="C363" t="n">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D363" t="n">
         <v>6</v>
@@ -6252,7 +6252,7 @@
         <v>1782.88</v>
       </c>
       <c r="C364" t="n">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D364" t="n">
         <v>6</v>
@@ -6284,7 +6284,7 @@
         <v>1857.91</v>
       </c>
       <c r="C366" t="n">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D366" t="n">
         <v>6</v>
@@ -6300,7 +6300,7 @@
         <v>1651.26</v>
       </c>
       <c r="C367" t="n">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D367" t="n">
         <v>5</v>
@@ -6316,7 +6316,7 @@
         <v>1786.63</v>
       </c>
       <c r="C368" t="n">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D368" t="n">
         <v>6</v>
@@ -6364,7 +6364,7 @@
         <v>1606.05</v>
       </c>
       <c r="C371" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D371" t="n">
         <v>9</v>
@@ -6380,7 +6380,7 @@
         <v>1746.99</v>
       </c>
       <c r="C372" t="n">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D372" t="n">
         <v>3</v>
@@ -6396,7 +6396,7 @@
         <v>1668.68</v>
       </c>
       <c r="C373" t="n">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D373" t="n">
         <v>2</v>
@@ -6412,7 +6412,7 @@
         <v>1574.48</v>
       </c>
       <c r="C374" t="n">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D374" t="n">
         <v>3</v>
@@ -6428,7 +6428,7 @@
         <v>1700.78</v>
       </c>
       <c r="C375" t="n">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D375" t="n">
         <v>8</v>
@@ -6444,7 +6444,7 @@
         <v>1703.84</v>
       </c>
       <c r="C376" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D376" t="n">
         <v>3</v>
@@ -6460,7 +6460,7 @@
         <v>1561.45</v>
       </c>
       <c r="C377" t="n">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D377" t="n">
         <v>4</v>
@@ -6476,7 +6476,7 @@
         <v>1501.49</v>
       </c>
       <c r="C378" t="n">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D378" t="n">
         <v>2</v>
@@ -6492,7 +6492,7 @@
         <v>1485.34</v>
       </c>
       <c r="C379" t="n">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D379" t="n">
         <v>2</v>
@@ -6540,7 +6540,7 @@
         <v>1325.5</v>
       </c>
       <c r="C382" t="n">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D382" t="n">
         <v>7</v>
@@ -6556,7 +6556,7 @@
         <v>1621.24</v>
       </c>
       <c r="C383" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D383" t="n">
         <v>5</v>
@@ -6588,7 +6588,7 @@
         <v>1285.44</v>
       </c>
       <c r="C385" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D385" t="n">
         <v>4</v>
@@ -6604,7 +6604,7 @@
         <v>1347.73</v>
       </c>
       <c r="C386" t="n">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D386" t="n">
         <v>9</v>
@@ -6620,7 +6620,7 @@
         <v>1266.38</v>
       </c>
       <c r="C387" t="n">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D387" t="n">
         <v>6</v>

</xml_diff>